<commit_message>
Add new updates of code
</commit_message>
<xml_diff>
--- a/CQ_Generation_Framework/output/domain_info.xlsx
+++ b/CQ_Generation_Framework/output/domain_info.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="62">
   <si>
     <t>MAIN_DOMAIN_NAME</t>
   </si>
@@ -46,52 +46,52 @@
     <t>Animal Models</t>
   </si>
   <si>
-    <t>Experimental Design</t>
-  </si>
-  <si>
-    <t>Treatment Protocols</t>
-  </si>
-  <si>
-    <t>Subject Characteristics</t>
-  </si>
-  <si>
-    <t>Laboratory Findings</t>
-  </si>
-  <si>
-    <t>Outcome Measures</t>
+    <t>Tumor Response</t>
+  </si>
+  <si>
+    <t>Healthy Tissue</t>
+  </si>
+  <si>
+    <t>Experimental Data</t>
   </si>
   <si>
     <t>Data Integration</t>
   </si>
   <si>
-    <t>Semantic Interoperability</t>
-  </si>
-  <si>
-    <t>Knowledge Graphs</t>
-  </si>
-  <si>
-    <t>FAIR Data Principles</t>
-  </si>
-  <si>
-    <t>Biomedical Research</t>
+    <t>SEND Standard</t>
+  </si>
+  <si>
+    <t>Clinical Observations</t>
+  </si>
+  <si>
+    <t>Laboratory Measurements</t>
+  </si>
+  <si>
+    <t>Intervention Procedures</t>
+  </si>
+  <si>
+    <t>Cohort Descriptions</t>
+  </si>
+  <si>
+    <t>Semantic Framework</t>
+  </si>
+  <si>
+    <t>Biomedical Knowledge Graphs</t>
+  </si>
+  <si>
+    <t>Data Standardization</t>
   </si>
   <si>
     <t>Translational Research</t>
   </si>
   <si>
-    <t>Complex Semantic Queries</t>
+    <t>FAIR Data Practices</t>
   </si>
   <si>
     <t>Data Annotation</t>
   </si>
   <si>
-    <t>Experimental Data</t>
-  </si>
-  <si>
-    <t>Radiotherapy Studies</t>
-  </si>
-  <si>
-    <t>Observational Studies</t>
+    <t>Research Collaboration</t>
   </si>
   <si>
     <t>Data Sharing</t>
@@ -109,88 +109,97 @@
     <t>trials</t>
   </si>
   <si>
-    <t>experiments</t>
-  </si>
-  <si>
     <t>animal</t>
   </si>
   <si>
     <t>models</t>
   </si>
   <si>
-    <t>design</t>
-  </si>
-  <si>
-    <t>treatment</t>
-  </si>
-  <si>
-    <t>characteristics</t>
+    <t>tumor</t>
+  </si>
+  <si>
+    <t>tissue</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>integration</t>
+  </si>
+  <si>
+    <t>SEND</t>
   </si>
   <si>
     <t>observations</t>
   </si>
   <si>
-    <t>findings</t>
-  </si>
-  <si>
-    <t>outcomes</t>
-  </si>
-  <si>
-    <t>data</t>
-  </si>
-  <si>
-    <t>integration</t>
-  </si>
-  <si>
-    <t>interoperability</t>
-  </si>
-  <si>
-    <t>queries</t>
-  </si>
-  <si>
-    <t>discovery</t>
+    <t>measurements</t>
+  </si>
+  <si>
+    <t>interventions</t>
+  </si>
+  <si>
+    <t>procedures</t>
+  </si>
+  <si>
+    <t>cohorts</t>
+  </si>
+  <si>
+    <t>semantic</t>
+  </si>
+  <si>
+    <t>bioinformatics</t>
   </si>
   <si>
     <t>research</t>
   </si>
   <si>
-    <t>bioinformatics</t>
-  </si>
-  <si>
-    <t>ontology</t>
+    <t>translational</t>
+  </si>
+  <si>
+    <t>FAIR</t>
+  </si>
+  <si>
+    <t>annotation</t>
+  </si>
+  <si>
+    <t>standardization</t>
+  </si>
+  <si>
+    <t>collaboration</t>
+  </si>
+  <si>
+    <t>sharing</t>
+  </si>
+  <si>
+    <t>analytics</t>
   </si>
   <si>
     <t>knowledge</t>
   </si>
   <si>
-    <t>graphs</t>
-  </si>
-  <si>
-    <t>FAIR</t>
-  </si>
-  <si>
-    <t>translational</t>
-  </si>
-  <si>
-    <t>annotation</t>
-  </si>
-  <si>
-    <t>studies</t>
-  </si>
-  <si>
-    <t>laboratories</t>
-  </si>
-  <si>
-    <t>semantic</t>
+    <t>graph</t>
+  </si>
+  <si>
+    <t>experimentation</t>
   </si>
   <si>
     <t>Preclinical Research</t>
   </si>
   <si>
-    <t>Radiation Treatment</t>
-  </si>
-  <si>
-    <t>Outcome Measurement</t>
+    <t>Radiation Effects</t>
+  </si>
+  <si>
+    <t>Animal Demographics</t>
+  </si>
+  <si>
+    <t>Interventions and Procedures</t>
+  </si>
+  <si>
+    <t>Temporal Information</t>
+  </si>
+  <si>
+    <t>Semantic Integration</t>
   </si>
 </sst>
 </file>
@@ -562,7 +571,7 @@
         <v>56</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -579,7 +588,7 @@
         <v>57</v>
       </c>
       <c r="F3" t="s">
-        <v>22</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -590,10 +599,10 @@
         <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F4" t="s">
-        <v>58</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -603,8 +612,11 @@
       <c r="C5" t="s">
         <v>30</v>
       </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -615,7 +627,7 @@
         <v>31</v>
       </c>
       <c r="F6" t="s">
-        <v>16</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -625,6 +637,9 @@
       <c r="C7" t="s">
         <v>32</v>
       </c>
+      <c r="F7" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="8" spans="1:6">
       <c r="B8" t="s">
@@ -633,6 +648,9 @@
       <c r="C8" t="s">
         <v>33</v>
       </c>
+      <c r="F8" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="9" spans="1:6">
       <c r="B9" t="s">
@@ -641,6 +659,9 @@
       <c r="C9" t="s">
         <v>34</v>
       </c>
+      <c r="F9" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="10" spans="1:6">
       <c r="B10" t="s">
@@ -648,6 +669,9 @@
       </c>
       <c r="C10" t="s">
         <v>35</v>
+      </c>
+      <c r="F10" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:6">

</xml_diff>